<commit_message>
Added Case IDs to openai table.
</commit_message>
<xml_diff>
--- a/openai/openai_ebola_europe_usa.xlsx
+++ b/openai/openai_ebola_europe_usa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lsh1604011/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/Documents/Ebola/ebola-importation/openai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B934F99D-A2F9-5D4A-95E3-767F00B98A74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A824FC2-0222-3C4C-B8FF-44C0519A76B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20620" yWindow="4980" windowWidth="36900" windowHeight="12660" xr2:uid="{DF932043-AF21-2D4D-92C9-63B815783400}"/>
+    <workbookView xWindow="19700" yWindow="3300" windowWidth="14720" windowHeight="12460" xr2:uid="{DF932043-AF21-2D4D-92C9-63B815783400}"/>
   </bookViews>
   <sheets>
     <sheet name="Europe" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="194">
   <si>
     <t>Year</t>
   </si>
@@ -620,6 +620,9 @@
   </si>
   <si>
     <t>For most European imported responder cases, the “travel measure” that mattered most was dedicated isolation transport, not airport passenger screening</t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -991,646 +994,706 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF2D41C-3E42-D044-A682-A0BBE6B18693}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
         <v>1976</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>17</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
         <v>1994</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>24</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>25</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2014</v>
-      </c>
-      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>2014</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>30</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>31</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>32</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>33</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>2014</v>
-      </c>
-      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>2014</v>
+      </c>
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>35</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>37</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>38</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>39</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>17</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>2014</v>
-      </c>
-      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2014</v>
+      </c>
+      <c r="C6" t="s">
         <v>40</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>41</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>42</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>44</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>39</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>45</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>2014</v>
-      </c>
-      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2014</v>
+      </c>
+      <c r="C7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>47</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>48</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>29</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>49</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>50</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>39</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>45</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>2014</v>
-      </c>
-      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>2014</v>
+      </c>
+      <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>27</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>28</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>36</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>30</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>51</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>52</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>33</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>2014</v>
-      </c>
-      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>2014</v>
+      </c>
+      <c r="C9" t="s">
         <v>53</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>54</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>55</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>36</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>56</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>57</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>39</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>45</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>2014</v>
-      </c>
-      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>2014</v>
+      </c>
+      <c r="C10" t="s">
         <v>26</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>58</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>59</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>30</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>61</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>62</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>17</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>2014</v>
-      </c>
-      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>2014</v>
+      </c>
+      <c r="C11" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>63</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>36</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>65</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>66</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>39</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>45</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>2014</v>
-      </c>
-      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>2014</v>
+      </c>
+      <c r="C12" t="s">
         <v>40</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>67</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>29</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>69</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>70</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>71</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>33</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>2014</v>
-      </c>
-      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>2014</v>
+      </c>
+      <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>72</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>73</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>36</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>49</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>74</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>39</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>45</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>2014</v>
-      </c>
-      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>2014</v>
+      </c>
+      <c r="C14" t="s">
         <v>18</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>75</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>76</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>36</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>77</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>78</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>39</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>45</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>2014</v>
-      </c>
-      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>2014</v>
+      </c>
+      <c r="C15" t="s">
         <v>79</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>80</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>81</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>36</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>82</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>84</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>85</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>2014</v>
-      </c>
-      <c r="B16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>2014</v>
+      </c>
+      <c r="C16" t="s">
         <v>86</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>87</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>88</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>29</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>89</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>90</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>91</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>45</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>2014</v>
-      </c>
-      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>2014</v>
+      </c>
+      <c r="C17" t="s">
         <v>10</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>92</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>93</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>36</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>94</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>95</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>96</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>97</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
         <v>2015</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>10</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>98</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>99</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>36</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>37</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>100</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>39</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>45</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
         <v>2015</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>79</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>101</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>102</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>103</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>104</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>105</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>106</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>85</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
         <v>2026</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>40</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>107</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>108</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>109</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>110</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>111</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>112</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>113</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>12</v>
       </c>
     </row>
@@ -1641,390 +1704,426 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7879EA13-E1E7-8640-B345-433083F7A6EA}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>114</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>2014</v>
-      </c>
-      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>2014</v>
+      </c>
+      <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>116</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>117</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>29</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>118</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>119</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>39</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>45</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>2014</v>
-      </c>
-      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3">
+        <v>2014</v>
+      </c>
+      <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>120</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>121</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>29</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>118</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>122</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>39</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>45</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>2014</v>
-      </c>
-      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4">
+        <v>2014</v>
+      </c>
+      <c r="C4" t="s">
         <v>115</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>123</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>124</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>125</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>126</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>127</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>39</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>45</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>2014</v>
-      </c>
-      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>2014</v>
+      </c>
+      <c r="C5" t="s">
         <v>115</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>128</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>129</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>130</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>118</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>131</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>39</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>45</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>2014</v>
-      </c>
-      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6">
+        <v>2014</v>
+      </c>
+      <c r="C6" t="s">
         <v>115</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>132</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>133</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>134</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>135</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>136</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>137</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>33</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>2014</v>
-      </c>
-      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7">
+        <v>2014</v>
+      </c>
+      <c r="C7" t="s">
         <v>115</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>138</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>139</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>140</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>141</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>142</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>143</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>45</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>2014</v>
-      </c>
-      <c r="B8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8">
+        <v>2014</v>
+      </c>
+      <c r="C8" t="s">
         <v>115</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>144</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>139</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>140</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>145</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>146</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>143</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>45</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>2014</v>
-      </c>
-      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9">
+        <v>2014</v>
+      </c>
+      <c r="C9" t="s">
         <v>115</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>147</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>148</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>29</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>126</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>149</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>150</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>45</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>2014</v>
-      </c>
-      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10">
+        <v>2014</v>
+      </c>
+      <c r="C10" t="s">
         <v>115</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>151</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>152</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>153</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>154</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>155</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>156</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>45</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11">
-        <v>2014</v>
-      </c>
-      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11">
+        <v>2014</v>
+      </c>
+      <c r="C11" t="s">
         <v>115</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>157</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>158</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>36</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>126</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>159</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>39</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>33</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12">
+        <v>30</v>
+      </c>
+      <c r="B12">
         <v>2015</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>115</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>160</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>161</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>36</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>162</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>163</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>39</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>45</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>17</v>
       </c>
     </row>

</xml_diff>